<commit_message>
Make Bill Rate OT a manual yellow input (blank/0 = auto)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JYNeTXzf1LDgiPyvKeRmyX
</commit_message>
<xml_diff>
--- a/Soloh_Travel_Pay_Package_Calculator_v1.1_18Load-18GP.xlsx
+++ b/Soloh_Travel_Pay_Package_Calculator_v1.1_18Load-18GP.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="172">
   <si>
     <t xml:space="preserve">Soloh Travel Pay Package Calculator v1.1   |   18% Load on W2 · No Onboarding Cost · 18% Desired GP</t>
   </si>
@@ -124,10 +124,7 @@
     <t xml:space="preserve">Client Contract Details</t>
   </si>
   <si>
-    <t xml:space="preserve">Bill Rate OT (Over Time)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT Override (Candidate)</t>
+    <t xml:space="preserve">Bill Rate OT (Over Time)  – 0 = auto</t>
   </si>
   <si>
     <t xml:space="preserve">- W2 Hourly Comp (RT)</t>
@@ -148,6 +145,9 @@
     <t xml:space="preserve">Expected hours per week</t>
   </si>
   <si>
+    <t xml:space="preserve">Bill Rate OT USED</t>
+  </si>
+  <si>
     <t xml:space="preserve">- Bonus / Reimbursement (W2)</t>
   </si>
   <si>
@@ -443,6 +443,9 @@
   </si>
   <si>
     <t xml:space="preserve">    ws.Range("D11").Value = 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ws.Range("D12").Value = 0   ' Bill Rate OT (0 = auto)</t>
   </si>
   <si>
     <t xml:space="preserve">    ws.Range("D13").Value = 0</t>
@@ -1122,16 +1125,16 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="169" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="5" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1927,7 +1930,7 @@
       </c>
       <c r="K10" s="16"/>
       <c r="L10" s="34" t="n">
-        <f aca="false">IF(D16="Yes",MIN(D22,IFERROR(INDEX(Lists!$G$1:$G$2,MATCH(D18,Lists!$F$1:$F$2,0)),40)),D22)*D11</f>
+        <f aca="false">IF(OR(D16="Yes",D12&gt;0),MIN(D22,IFERROR(INDEX(Lists!$G$1:$G$2,MATCH(D18,Lists!$F$1:$F$2,0)),40)),D22)*D11</f>
         <v>3240</v>
       </c>
       <c r="M10" s="35" t="n">
@@ -1975,7 +1978,7 @@
       </c>
       <c r="K11" s="16"/>
       <c r="L11" s="34" t="n">
-        <f aca="false">(D22-IF(D16="Yes",MIN(D22,IFERROR(INDEX(Lists!$G$1:$G$2,MATCH(D18,Lists!$F$1:$F$2,0)),40)),D22))*D12</f>
+        <f aca="false">(D22-IF(OR(D16="Yes",D12&gt;0),MIN(D22,IFERROR(INDEX(Lists!$G$1:$G$2,MATCH(D18,Lists!$F$1:$F$2,0)),40)),D22))*D14</f>
         <v>0</v>
       </c>
       <c r="M11" s="35" t="n">
@@ -2007,19 +2010,16 @@
         <v>32</v>
       </c>
       <c r="C12" s="14"/>
-      <c r="D12" s="26" t="n">
-        <f aca="false">D11*IF(D16="Yes",IFERROR(INDEX(Lists!$E$1:$E$4,MATCH(D17,Lists!$D$1:$D$4,0)),1),1)</f>
-        <v>90</v>
+      <c r="D12" s="22" t="n">
+        <v>0</v>
       </c>
       <c r="E12" s="1"/>
-      <c r="F12" s="38" t="s">
-        <v>33</v>
-      </c>
-      <c r="G12" s="38"/>
-      <c r="H12" s="38"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="19"/>
       <c r="I12" s="1"/>
       <c r="J12" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K12" s="16"/>
       <c r="L12" s="34" t="n">
@@ -2032,11 +2032,11 @@
       </c>
       <c r="N12" s="1"/>
       <c r="O12" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P12" s="12"/>
       <c r="Q12" s="12"/>
-      <c r="R12" s="39" t="n">
+      <c r="R12" s="38" t="n">
         <f aca="false">D21</f>
         <v>13</v>
       </c>
@@ -2055,23 +2055,23 @@
     <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
       <c r="B13" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="33" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="1"/>
-      <c r="F13" s="40" t="s">
-        <v>37</v>
-      </c>
-      <c r="G13" s="40"/>
+      <c r="F13" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13" s="39"/>
       <c r="H13" s="22" t="n">
         <v>0</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="K13" s="16"/>
       <c r="L13" s="34" t="n">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="N13" s="1"/>
       <c r="O13" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P13" s="12"/>
       <c r="Q13" s="12"/>
-      <c r="R13" s="39" t="n">
+      <c r="R13" s="38" t="n">
         <f aca="false">D22</f>
         <v>36</v>
       </c>
@@ -2106,12 +2106,17 @@
     </row>
     <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="19"/>
+      <c r="B14" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="14"/>
+      <c r="D14" s="36" t="n">
+        <f aca="false">IF(D12&gt;0,D12,D11*IF(D16="Yes",IFERROR(INDEX(Lists!$E$1:$E$4,MATCH(D17,Lists!$D$1:$D$4,0)),1),1))</f>
+        <v>90</v>
+      </c>
       <c r="E14" s="1"/>
-      <c r="F14" s="40"/>
-      <c r="G14" s="40"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="39"/>
       <c r="H14" s="22"/>
       <c r="I14" s="1"/>
       <c r="J14" s="16" t="s">
@@ -2132,7 +2137,7 @@
       </c>
       <c r="P14" s="12"/>
       <c r="Q14" s="12"/>
-      <c r="R14" s="39" t="n">
+      <c r="R14" s="38" t="n">
         <f aca="false">D23</f>
         <v>12</v>
       </c>
@@ -2199,11 +2204,11 @@
         <v>45</v>
       </c>
       <c r="E16" s="1"/>
-      <c r="F16" s="38" t="s">
+      <c r="F16" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="G16" s="38"/>
-      <c r="H16" s="38"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="40"/>
       <c r="I16" s="1"/>
       <c r="J16" s="41" t="s">
         <v>47</v>
@@ -2413,7 +2418,7 @@
     <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
       <c r="B21" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C21" s="14"/>
       <c r="D21" s="47" t="n">
@@ -2463,7 +2468,7 @@
     <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
       <c r="B22" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="47" t="n">
@@ -3171,7 +3176,7 @@
     </row>
   </sheetData>
   <sheetProtection sheet="true" password="c784"/>
-  <mergeCells count="57">
+  <mergeCells count="56">
     <mergeCell ref="J3:M3"/>
     <mergeCell ref="O3:R3"/>
     <mergeCell ref="B5:D5"/>
@@ -3187,7 +3192,6 @@
     <mergeCell ref="J10:K10"/>
     <mergeCell ref="J11:K11"/>
     <mergeCell ref="O11:R11"/>
-    <mergeCell ref="F12:H12"/>
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="O12:Q12"/>
     <mergeCell ref="F13:G14"/>
@@ -3547,7 +3551,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A53"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="140"/>
@@ -3662,12 +3666,12 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="70" t="s">
+      <c r="A24" s="71" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="71" t="s">
+      <c r="A25" s="70" t="s">
         <v>145</v>
       </c>
     </row>
@@ -3687,12 +3691,12 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="70" t="s">
+      <c r="A29" s="71" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="71" t="s">
+      <c r="A30" s="70" t="s">
         <v>150</v>
       </c>
     </row>
@@ -3717,12 +3721,12 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="70" t="s">
+      <c r="A35" s="71" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="71" t="s">
+      <c r="A36" s="70" t="s">
         <v>156</v>
       </c>
     </row>
@@ -3752,12 +3756,12 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="71"/>
+      <c r="A42" s="71" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="71" t="s">
-        <v>162</v>
-      </c>
+      <c r="A43" s="71"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="71" t="s">
@@ -3766,12 +3770,12 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="71" t="s">
-        <v>130</v>
+        <v>164</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="71" t="s">
-        <v>164</v>
+        <v>130</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3806,7 +3810,12 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="71" t="s">
-        <v>161</v>
+        <v>171</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="71" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>